<commit_message>
Headers for the spreadsheet and remove empty cells
</commit_message>
<xml_diff>
--- a/output/parts.xlsx
+++ b/output/parts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="134">
   <si>
     <t>ID</t>
   </si>
@@ -221,11 +221,7 @@
     <t>16.0 x 13.97 deep</t>
   </si>
   <si>
-    <t>30.0
--</t>
-  </si>
-  <si>
-    <t>-</t>
+    <t>30.0</t>
   </si>
   <si>
     <t>0.626"</t>
@@ -237,9 +233,6 @@
     <t>0.630" x 0.550" deep</t>
   </si>
   <si>
-    <t>30.0</t>
-  </si>
-  <si>
     <t>30X_cb_A_B_.nc</t>
   </si>
   <si>
@@ -291,8 +284,7 @@
     <t>20.1168 x 17.399 deep</t>
   </si>
   <si>
-    <t>40.0
--</t>
+    <t>40.0</t>
   </si>
   <si>
     <t>0.855"</t>
@@ -302,9 +294,6 @@
   </si>
   <si>
     <t>0.792" x 0.685" deep</t>
-  </si>
-  <si>
-    <t>40.0</t>
   </si>
   <si>
     <t>40X_cb_A_B_.nc</t>
@@ -469,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O97"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="8.31640625" customWidth="true" bestFit="true"/>
@@ -480,6 +469,10 @@
     <col min="6" max="6" width="7.80078125" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="24.03125" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="5.87109375" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="7.26171875" customWidth="true" bestFit="true"/>
+    <col min="10" max="10" width="7.80078125" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="17.73828125" customWidth="true" bestFit="true"/>
+    <col min="12" max="12" width="5.87109375" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -507,6 +500,18 @@
       <c r="H1" t="s" s="0">
         <v>7</v>
       </c>
+      <c r="I1" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>5</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
@@ -1577,22 +1582,13 @@
         <v>70</v>
       </c>
       <c r="J42" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K42" t="s" s="0">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L42" t="s" s="0">
-        <v>71</v>
-      </c>
-      <c r="M42" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="N42" t="s" s="0">
-        <v>73</v>
-      </c>
-      <c r="O42" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43">
@@ -1600,7 +1596,7 @@
         <v>63</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C43" t="s" s="0">
         <v>65</v>
@@ -1624,22 +1620,13 @@
         <v>70</v>
       </c>
       <c r="J43" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K43" t="s" s="0">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L43" t="s" s="0">
-        <v>71</v>
-      </c>
-      <c r="M43" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="N43" t="s" s="0">
-        <v>73</v>
-      </c>
-      <c r="O43" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="44">
@@ -1647,7 +1634,7 @@
         <v>63</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C44" t="s" s="0">
         <v>65</v>
@@ -1671,22 +1658,13 @@
         <v>70</v>
       </c>
       <c r="J44" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K44" t="s" s="0">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L44" t="s" s="0">
-        <v>71</v>
-      </c>
-      <c r="M44" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="N44" t="s" s="0">
-        <v>73</v>
-      </c>
-      <c r="O44" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="45">
@@ -1694,7 +1672,7 @@
         <v>63</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C45" t="s" s="0">
         <v>65</v>
@@ -1718,22 +1696,13 @@
         <v>70</v>
       </c>
       <c r="J45" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K45" t="s" s="0">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="L45" t="s" s="0">
-        <v>71</v>
-      </c>
-      <c r="M45" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="N45" t="s" s="0">
-        <v>73</v>
-      </c>
-      <c r="O45" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="46">
@@ -1756,10 +1725,10 @@
         <v>67</v>
       </c>
       <c r="G46" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H46" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47">
@@ -1767,7 +1736,7 @@
         <v>63</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C47" t="s" s="0">
         <v>65</v>
@@ -1782,10 +1751,10 @@
         <v>67</v>
       </c>
       <c r="G47" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H47" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="48">
@@ -1808,10 +1777,10 @@
         <v>67</v>
       </c>
       <c r="G48" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H48" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49">
@@ -1819,7 +1788,7 @@
         <v>63</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C49" t="s" s="0">
         <v>65</v>
@@ -1834,10 +1803,10 @@
         <v>67</v>
       </c>
       <c r="G49" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H49" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50">
@@ -1860,10 +1829,10 @@
         <v>67</v>
       </c>
       <c r="G50" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H50" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="51">
@@ -1871,7 +1840,7 @@
         <v>63</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C51" t="s" s="0">
         <v>65</v>
@@ -1886,10 +1855,10 @@
         <v>67</v>
       </c>
       <c r="G51" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H51" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52">
@@ -1912,10 +1881,10 @@
         <v>67</v>
       </c>
       <c r="G52" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H52" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="53">
@@ -1923,7 +1892,7 @@
         <v>63</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C53" t="s" s="0">
         <v>65</v>
@@ -1938,10 +1907,10 @@
         <v>67</v>
       </c>
       <c r="G53" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H53" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="54">
@@ -1964,10 +1933,10 @@
         <v>67</v>
       </c>
       <c r="G54" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H54" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55">
@@ -1975,7 +1944,7 @@
         <v>63</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C55" t="s" s="0">
         <v>65</v>
@@ -1990,10 +1959,10 @@
         <v>67</v>
       </c>
       <c r="G55" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H55" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="56">
@@ -2016,10 +1985,10 @@
         <v>67</v>
       </c>
       <c r="G56" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H56" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="57">
@@ -2027,7 +1996,7 @@
         <v>63</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C57" t="s" s="0">
         <v>65</v>
@@ -2042,10 +2011,10 @@
         <v>67</v>
       </c>
       <c r="G57" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H57" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="58">
@@ -2068,10 +2037,10 @@
         <v>67</v>
       </c>
       <c r="G58" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H58" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="59">
@@ -2079,7 +2048,7 @@
         <v>63</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C59" t="s" s="0">
         <v>65</v>
@@ -2094,10 +2063,10 @@
         <v>67</v>
       </c>
       <c r="G59" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H59" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="60">
@@ -2120,10 +2089,10 @@
         <v>67</v>
       </c>
       <c r="G60" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H60" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="61">
@@ -2131,7 +2100,7 @@
         <v>63</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C61" t="s" s="0">
         <v>65</v>
@@ -2146,18 +2115,18 @@
         <v>67</v>
       </c>
       <c r="G61" t="s" s="0">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H61" t="s" s="0">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B62" t="s" s="0">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C62" t="s" s="0">
         <v>65</v>
@@ -2166,45 +2135,36 @@
         <v>11</v>
       </c>
       <c r="E62" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="F62" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G62" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="F62" t="s" s="0">
+      <c r="H62" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="G62" t="s" s="0">
+      <c r="I62" t="s" s="0">
         <v>91</v>
       </c>
-      <c r="H62" t="s" s="0">
+      <c r="J62" t="s" s="0">
         <v>92</v>
       </c>
-      <c r="I62" t="s" s="0">
-        <v>70</v>
-      </c>
-      <c r="J62" t="s" s="0">
-        <v>70</v>
-      </c>
       <c r="K62" t="s" s="0">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="L62" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="M62" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="N62" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="O62" t="s" s="0">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B63" t="s" s="0">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C63" t="s" s="0">
         <v>65</v>
@@ -2213,45 +2173,36 @@
         <v>11</v>
       </c>
       <c r="E63" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="F63" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G63" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="F63" t="s" s="0">
+      <c r="H63" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="G63" t="s" s="0">
+      <c r="I63" t="s" s="0">
         <v>91</v>
       </c>
-      <c r="H63" t="s" s="0">
+      <c r="J63" t="s" s="0">
         <v>92</v>
       </c>
-      <c r="I63" t="s" s="0">
-        <v>70</v>
-      </c>
-      <c r="J63" t="s" s="0">
-        <v>70</v>
-      </c>
       <c r="K63" t="s" s="0">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="L63" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="M63" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="N63" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="O63" t="s" s="0">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B64" t="s" s="0">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C64" t="s" s="0">
         <v>65</v>
@@ -2260,45 +2211,36 @@
         <v>11</v>
       </c>
       <c r="E64" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="F64" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G64" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="F64" t="s" s="0">
+      <c r="H64" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="G64" t="s" s="0">
+      <c r="I64" t="s" s="0">
         <v>91</v>
       </c>
-      <c r="H64" t="s" s="0">
+      <c r="J64" t="s" s="0">
         <v>92</v>
       </c>
-      <c r="I64" t="s" s="0">
-        <v>70</v>
-      </c>
-      <c r="J64" t="s" s="0">
-        <v>70</v>
-      </c>
       <c r="K64" t="s" s="0">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="L64" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="M64" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="N64" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="O64" t="s" s="0">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B65" t="s" s="0">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C65" t="s" s="0">
         <v>65</v>
@@ -2307,45 +2249,36 @@
         <v>11</v>
       </c>
       <c r="E65" t="s" s="0">
+        <v>87</v>
+      </c>
+      <c r="F65" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G65" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="F65" t="s" s="0">
+      <c r="H65" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="G65" t="s" s="0">
+      <c r="I65" t="s" s="0">
         <v>91</v>
       </c>
-      <c r="H65" t="s" s="0">
+      <c r="J65" t="s" s="0">
         <v>92</v>
       </c>
-      <c r="I65" t="s" s="0">
-        <v>70</v>
-      </c>
-      <c r="J65" t="s" s="0">
-        <v>70</v>
-      </c>
       <c r="K65" t="s" s="0">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="L65" t="s" s="0">
-        <v>93</v>
-      </c>
-      <c r="M65" t="s" s="0">
-        <v>94</v>
-      </c>
-      <c r="N65" t="s" s="0">
-        <v>95</v>
-      </c>
-      <c r="O65" t="s" s="0">
-        <v>96</v>
+        <v>90</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C66" t="s" s="0">
         <v>65</v>
@@ -2354,24 +2287,24 @@
         <v>20</v>
       </c>
       <c r="E66" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F66" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G66" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H66" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F66" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G66" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H66" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B67" t="s" s="0">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C67" t="s" s="0">
         <v>65</v>
@@ -2380,24 +2313,24 @@
         <v>20</v>
       </c>
       <c r="E67" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F67" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G67" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H67" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F67" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G67" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H67" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B68" t="s" s="0">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C68" t="s" s="0">
         <v>65</v>
@@ -2406,24 +2339,24 @@
         <v>20</v>
       </c>
       <c r="E68" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F68" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G68" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H68" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F68" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G68" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H68" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B69" t="s" s="0">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C69" t="s" s="0">
         <v>65</v>
@@ -2432,24 +2365,24 @@
         <v>20</v>
       </c>
       <c r="E69" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F69" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G69" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H69" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F69" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G69" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H69" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B70" t="s" s="0">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C70" t="s" s="0">
         <v>65</v>
@@ -2458,24 +2391,24 @@
         <v>20</v>
       </c>
       <c r="E70" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F70" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G70" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H70" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F70" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G70" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H70" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B71" t="s" s="0">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C71" t="s" s="0">
         <v>65</v>
@@ -2484,24 +2417,24 @@
         <v>20</v>
       </c>
       <c r="E71" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F71" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G71" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H71" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F71" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G71" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H71" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B72" t="s" s="0">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C72" t="s" s="0">
         <v>65</v>
@@ -2510,24 +2443,24 @@
         <v>20</v>
       </c>
       <c r="E72" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F72" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G72" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H72" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F72" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G72" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H72" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B73" t="s" s="0">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C73" t="s" s="0">
         <v>65</v>
@@ -2536,24 +2469,24 @@
         <v>20</v>
       </c>
       <c r="E73" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F73" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G73" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H73" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F73" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G73" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H73" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B74" t="s" s="0">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C74" t="s" s="0">
         <v>65</v>
@@ -2562,24 +2495,24 @@
         <v>20</v>
       </c>
       <c r="E74" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F74" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G74" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H74" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F74" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G74" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H74" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B75" t="s" s="0">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C75" t="s" s="0">
         <v>65</v>
@@ -2588,24 +2521,24 @@
         <v>20</v>
       </c>
       <c r="E75" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F75" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G75" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H75" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F75" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G75" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H75" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B76" t="s" s="0">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C76" t="s" s="0">
         <v>65</v>
@@ -2614,24 +2547,24 @@
         <v>20</v>
       </c>
       <c r="E76" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F76" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G76" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H76" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F76" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G76" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H76" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B77" t="s" s="0">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C77" t="s" s="0">
         <v>65</v>
@@ -2640,24 +2573,24 @@
         <v>20</v>
       </c>
       <c r="E77" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F77" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G77" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H77" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F77" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G77" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H77" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B78" t="s" s="0">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C78" t="s" s="0">
         <v>65</v>
@@ -2666,24 +2599,24 @@
         <v>20</v>
       </c>
       <c r="E78" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F78" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G78" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H78" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F78" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G78" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H78" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B79" t="s" s="0">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C79" t="s" s="0">
         <v>65</v>
@@ -2692,24 +2625,24 @@
         <v>20</v>
       </c>
       <c r="E79" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F79" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G79" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H79" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F79" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G79" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H79" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B80" t="s" s="0">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C80" t="s" s="0">
         <v>65</v>
@@ -2718,24 +2651,24 @@
         <v>20</v>
       </c>
       <c r="E80" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F80" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G80" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H80" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F80" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G80" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H80" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="0">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B81" t="s" s="0">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C81" t="s" s="0">
         <v>65</v>
@@ -2744,432 +2677,432 @@
         <v>20</v>
       </c>
       <c r="E81" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="F81" t="s" s="0">
+        <v>88</v>
+      </c>
+      <c r="G81" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="H81" t="s" s="0">
         <v>90</v>
-      </c>
-      <c r="F81" t="s" s="0">
-        <v>90</v>
-      </c>
-      <c r="G81" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="H81" t="s" s="0">
-        <v>96</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B82" t="s" s="0">
+        <v>115</v>
+      </c>
+      <c r="C82" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D82" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E82" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F82" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G82" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B82" t="s" s="0">
+      <c r="H82" t="s" s="0">
         <v>118</v>
-      </c>
-      <c r="C82" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D82" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E82" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F82" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G82" t="s" s="0">
-        <v>120</v>
-      </c>
-      <c r="H82" t="s" s="0">
-        <v>121</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="C83" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D83" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E83" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F83" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G83" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B83" t="s" s="0">
-        <v>122</v>
-      </c>
-      <c r="C83" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D83" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E83" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F83" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G83" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H83" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="C84" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D84" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E84" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F84" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G84" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B84" t="s" s="0">
-        <v>123</v>
-      </c>
-      <c r="C84" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D84" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E84" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F84" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G84" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H84" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>121</v>
+      </c>
+      <c r="C85" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D85" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E85" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F85" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G85" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B85" t="s" s="0">
-        <v>124</v>
-      </c>
-      <c r="C85" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D85" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E85" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F85" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G85" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H85" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>122</v>
+      </c>
+      <c r="C86" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D86" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E86" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F86" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G86" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B86" t="s" s="0">
-        <v>125</v>
-      </c>
-      <c r="C86" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D86" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E86" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F86" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G86" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H86" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B87" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="C87" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D87" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E87" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F87" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G87" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B87" t="s" s="0">
-        <v>126</v>
-      </c>
-      <c r="C87" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D87" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E87" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F87" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G87" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H87" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B88" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="C88" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D88" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E88" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F88" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G88" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B88" t="s" s="0">
-        <v>127</v>
-      </c>
-      <c r="C88" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D88" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E88" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F88" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G88" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H88" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B89" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="C89" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D89" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E89" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F89" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G89" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B89" t="s" s="0">
-        <v>128</v>
-      </c>
-      <c r="C89" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D89" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E89" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F89" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G89" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H89" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>126</v>
+      </c>
+      <c r="C90" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D90" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E90" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F90" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G90" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B90" t="s" s="0">
-        <v>129</v>
-      </c>
-      <c r="C90" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D90" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E90" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F90" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G90" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H90" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>127</v>
+      </c>
+      <c r="C91" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D91" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E91" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F91" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G91" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B91" t="s" s="0">
-        <v>130</v>
-      </c>
-      <c r="C91" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D91" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E91" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F91" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G91" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H91" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B92" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="C92" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D92" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E92" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F92" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G92" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B92" t="s" s="0">
-        <v>131</v>
-      </c>
-      <c r="C92" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D92" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E92" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F92" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G92" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H92" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B93" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="C93" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D93" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E93" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F93" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G93" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B93" t="s" s="0">
-        <v>132</v>
-      </c>
-      <c r="C93" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D93" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E93" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F93" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G93" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H93" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B94" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="C94" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D94" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E94" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F94" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G94" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B94" t="s" s="0">
-        <v>133</v>
-      </c>
-      <c r="C94" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D94" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E94" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F94" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G94" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H94" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B95" t="s" s="0">
+        <v>131</v>
+      </c>
+      <c r="C95" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D95" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E95" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F95" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G95" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B95" t="s" s="0">
-        <v>134</v>
-      </c>
-      <c r="C95" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D95" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E95" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F95" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G95" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H95" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B96" t="s" s="0">
+        <v>132</v>
+      </c>
+      <c r="C96" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D96" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E96" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F96" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G96" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B96" t="s" s="0">
-        <v>135</v>
-      </c>
-      <c r="C96" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D96" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E96" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F96" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G96" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H96" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B97" t="s" s="0">
+        <v>133</v>
+      </c>
+      <c r="C97" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="D97" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E97" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="F97" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="G97" t="s" s="0">
         <v>117</v>
       </c>
-      <c r="B97" t="s" s="0">
-        <v>136</v>
-      </c>
-      <c r="C97" t="s" s="0">
-        <v>65</v>
-      </c>
-      <c r="D97" t="s" s="0">
-        <v>20</v>
-      </c>
-      <c r="E97" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="F97" t="s" s="0">
-        <v>119</v>
-      </c>
-      <c r="G97" t="s" s="0">
-        <v>120</v>
-      </c>
       <c r="H97" t="s" s="0">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>